<commit_message>
Implemented TestNG XML - Smoke and Regression Test Suites
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/LoginData.xlsx
+++ b/src/main/resources/testdata/LoginData.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Archana\AutomationDemo\OrangeHRM_Automation\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BDD1E38-D86C-474C-86E5-AE0EB287B14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0A327D-9F7A-49F6-91A6-D37732E425EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
+    <sheet name="smoke" sheetId="4" r:id="rId1"/>
+    <sheet name="regression" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -43,9 +43,6 @@
     <t>ExpectedResult</t>
   </si>
   <si>
-    <t>locator</t>
-  </si>
-  <si>
     <t>Verify login with valid credentials</t>
   </si>
   <si>
@@ -67,9 +64,6 @@
     <t>To check screenshot is captued for failed tests</t>
   </si>
   <si>
-    <t>Negative</t>
-  </si>
-  <si>
     <t>Dashboard123</t>
   </si>
   <si>
@@ -107,16 +101,58 @@
   </si>
   <si>
     <t>ad123</t>
+  </si>
+  <si>
+    <t>Locator</t>
+  </si>
+  <si>
+    <t>TestCase_ID</t>
+  </si>
+  <si>
+    <t>Regression</t>
+  </si>
+  <si>
+    <t>Sanity</t>
+  </si>
+  <si>
+    <t>TC_Reg_1</t>
+  </si>
+  <si>
+    <t>TC_Reg_2</t>
+  </si>
+  <si>
+    <t>TC_Reg_3</t>
+  </si>
+  <si>
+    <t>TC_Smk_1</t>
+  </si>
+  <si>
+    <t>TC_Smk_2</t>
+  </si>
+  <si>
+    <t>TC_Reg_4</t>
+  </si>
+  <si>
+    <t>TC_Reg_5</t>
+  </si>
+  <si>
+    <t>TC_Reg_6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -440,56 +476,86 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE23C912-919E-4882-9CBF-0E92FC257660}">
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="71.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>7</v>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -499,115 +565,181 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44B3EB90-9EE7-4971-9850-AC5E93D3F67E}">
-  <dimension ref="A2:F6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="92.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="71.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="E7" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="F7" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
+      <c r="G7" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added sanity test suite xml
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/LoginData.xlsx
+++ b/src/main/resources/testdata/LoginData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Archana\AutomationDemo\OrangeHRM_Automation\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF0A327D-9F7A-49F6-91A6-D37732E425EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D144B42D-1177-4069-8844-E196B175344F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="smoke" sheetId="4" r:id="rId1"/>
     <sheet name="regression" sheetId="3" r:id="rId2"/>
+    <sheet name="sanity" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="37">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -136,7 +137,7 @@
     <t>TC_Reg_5</t>
   </si>
   <si>
-    <t>TC_Reg_6</t>
+    <t>TC_Neg_1</t>
   </si>
 </sst>
 </file>
@@ -565,7 +566,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44B3EB90-9EE7-4971-9850-AC5E93D3F67E}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -715,31 +716,69 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBEA5298-5A8B-48E9-B7A9-C5AD390FB830}">
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>